<commit_message>
Update KAILA Founder Presentation materials and financial model
- Revised content in multiple presentation files to reflect updated product descriptions and financial projections.
- Adjusted funding scenarios and financial model to align with lean pilot approach and revised budget estimates.
- Enhanced clarity on market assumptions and pilot execution strategies in investor package documents.
- Updated startup guide to streamline the initial pilot process and emphasize the importance of validation before software development.
</commit_message>
<xml_diff>
--- a/KAILA_Founder_Grade_Package/08_Three_Year_Financial_Projection.xlsx
+++ b/KAILA_Founder_Grade_Package/08_Three_Year_Financial_Projection.xlsx
@@ -962,7 +962,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>A manual version of the marketplace run with simple tools such as forms, spreadsheets, Facebook, and Messenger before building the full app.</t>
+          <t>A marketplace test using the existing browser MVP/native wrapper plus Facebook page posts, Messenger follow-up, and manual operations support.</t>
         </is>
       </c>
     </row>
@@ -1246,11 +1246,11 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>1500</v>
+        <v>500</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Estimated startup operating cost</t>
+          <t>Lean pilot: free tiers/current hosting where possible</t>
         </is>
       </c>
     </row>
@@ -1261,11 +1261,11 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>3000</v>
+        <v>1000</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Local social media and field recruitment</t>
+          <t>Facebook page, organic posting, small boosts only when needed</t>
         </is>
       </c>
     </row>
@@ -1276,11 +1276,11 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>5000</v>
+        <v>1000</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Part-time support or allowance</t>
+          <t>Founder-led operations; small allowance for field support</t>
         </is>
       </c>
     </row>
@@ -1291,11 +1291,11 @@
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Permits, documentation, miscellaneous</t>
+          <t>Defer formal admin spend during validation unless required</t>
         </is>
       </c>
     </row>
@@ -1306,11 +1306,11 @@
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>If SMS is used; can be 0 for Messenger-only pilot</t>
+          <t>Use in-app flow and Messenger during pilot</t>
         </is>
       </c>
     </row>
@@ -1325,7 +1325,7 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Founder-led development initially</t>
+          <t>Browser MVP and native wrapper already built; founder-led polish</t>
         </is>
       </c>
     </row>
@@ -4391,9 +4391,10 @@
           <t>Metric</t>
         </is>
       </c>
-      <c r="B2" s="13">
-        <f>'Assumptions'!B7</f>
-        <v/>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
       </c>
       <c r="C2" s="13" t="inlineStr">
         <is>
@@ -4408,7 +4409,7 @@
         </is>
       </c>
       <c r="B3" s="14">
-        <f>'Assumptions'!B8</f>
+        <f>'Assumptions'!B7</f>
         <v/>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -4424,7 +4425,7 @@
         </is>
       </c>
       <c r="B4" s="14">
-        <f>'Assumptions'!B7*'Assumptions'!B8</f>
+        <f>'Assumptions'!B8</f>
         <v/>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -4440,7 +4441,7 @@
         </is>
       </c>
       <c r="B5" s="14">
-        <f>'Assumptions'!B16</f>
+        <f>'Assumptions'!B7*'Assumptions'!B8</f>
         <v/>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -4456,7 +4457,7 @@
         </is>
       </c>
       <c r="B6" s="14">
-        <f>'Assumptions'!B6</f>
+        <f>'Assumptions'!B16</f>
         <v/>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -4472,7 +4473,7 @@
         </is>
       </c>
       <c r="B7" s="14">
-        <f>'Assumptions'!B16/'Assumptions'!B6</f>
+        <f>'Assumptions'!B6</f>
         <v/>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -4488,7 +4489,7 @@
         </is>
       </c>
       <c r="B8" s="14">
-        <f>('Assumptions'!B7*'Assumptions'!B8)-('Assumptions'!B16/'Assumptions'!B6)</f>
+        <f>IF(B7&gt;0,B6/B7,0)</f>
         <v/>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -4504,7 +4505,7 @@
         </is>
       </c>
       <c r="B9" s="14">
-        <f>IF(B8&gt;0,('Assumptions'!B12+'Assumptions'!B13+'Assumptions'!B14+'Assumptions'!B15+'Assumptions'!B17)/B8,0)</f>
+        <f>B5-B8</f>
         <v/>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -4520,7 +4521,7 @@
         </is>
       </c>
       <c r="B10" s="14">
-        <f>IF(B8&gt;0, ('Assumptions'!B12+'Assumptions'!B13+'Assumptions'!B14+'Assumptions'!B15+'Assumptions'!B17)/B8, "N/A")</f>
+        <f>IF(B9&gt;0,('Assumptions'!B12+'Assumptions'!B13+'Assumptions'!B14+'Assumptions'!B15+'Assumptions'!B17)/B9, "N/A")</f>
         <v/>
       </c>
       <c r="C10" s="3" t="inlineStr">

</xml_diff>